<commit_message>
test(fase-2): preservar tildes en el archivo de Excel
</commit_message>
<xml_diff>
--- a/tests/fixtures/catalog.xlsx
+++ b/tests/fixtures/catalog.xlsx
@@ -85,7 +85,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Prote?na de prueba</t>
+          <t>Proteína de prueba</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -100,7 +100,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Descripci?n actualizada</t>
+          <t>Descripción actualizada</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>